<commit_message>
Refactor - final sublineage set
</commit_message>
<xml_diff>
--- a/tabular/sublineage/herv_sublineage_data.xlsx
+++ b/tabular/sublineage/herv_sublineage_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rob/Projects/erv/locus-level/ERVdb-HomoSapiens/tabular/sublineage/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B828DC8D-DAFA-1845-860C-B35390FBC2C1}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EF21E09-0E87-0841-AC9B-43087069E310}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10520" yWindow="1380" windowWidth="23060" windowHeight="16200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2220" yWindow="860" windowWidth="23060" windowHeight="16200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="sublineage" sheetId="2" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1004" uniqueCount="235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1004" uniqueCount="236">
   <si>
     <t>sequenceID</t>
   </si>
@@ -736,6 +736,9 @@
   </si>
   <si>
     <t>ERVR-1.Zeta.W9P.P.G25</t>
+  </si>
+  <si>
+    <t>ERV-3.Lambda</t>
   </si>
 </sst>
 </file>
@@ -2933,7 +2936,7 @@
       </c>
       <c r="E19" s="2"/>
       <c r="F19" s="2" t="s">
-        <v>106</v>
+        <v>235</v>
       </c>
       <c r="G19" s="2" t="s">
         <v>198</v>
@@ -3002,7 +3005,7 @@
       </c>
       <c r="E20" s="3"/>
       <c r="F20" s="2" t="s">
-        <v>106</v>
+        <v>235</v>
       </c>
       <c r="G20" s="2" t="s">
         <v>198</v>
@@ -3071,7 +3074,7 @@
       </c>
       <c r="E21" s="2"/>
       <c r="F21" s="2" t="s">
-        <v>106</v>
+        <v>235</v>
       </c>
       <c r="G21" s="2" t="s">
         <v>198</v>

</xml_diff>